<commit_message>
Wrote inspiration and similar section of documentation
</commit_message>
<xml_diff>
--- a/documentation/Time Plan.xlsx
+++ b/documentation/Time Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://collyer82-my.sharepoint.com/personal/25cookeg899_collyers_ac_uk/Documents/01 - Computer Science/Python Projects/Theatre-Booking/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{2D523807-7404-4E18-A3A7-2E609803194E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F67DFED9-50B2-4CEA-83FB-C3254BC2F593}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{2D523807-7404-4E18-A3A7-2E609803194E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3CDFC6B-1B1B-48B0-898B-2FDF5C8F19A5}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="3072" yWindow="3072" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t>Time Plan: Design and Develop a Theatre Booking System</t>
   </si>
@@ -112,6 +112,9 @@
   </si>
   <si>
     <t>UML (Pseudocode)</t>
+  </si>
+  <si>
+    <t>Week Ending</t>
   </si>
 </sst>
 </file>
@@ -314,9 +317,6 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -329,14 +329,17 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -357,6 +360,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -637,21 +644,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="11"/>
+      <c r="A2" s="23" t="s">
+        <v>23</v>
+      </c>
       <c r="B2" s="6">
         <v>46080</v>
       </c>
@@ -695,45 +704,45 @@
       <c r="J3" s="10"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
+      <c r="I4" s="13"/>
       <c r="J4" s="7"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
       <c r="J5" s="4"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="23"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
       <c r="J6" s="4"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
@@ -751,16 +760,16 @@
       <c r="J7" s="10"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="23"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
       <c r="I8" s="7"/>
       <c r="J8" s="7"/>
     </row>
@@ -768,13 +777,13 @@
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="23"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
     </row>
@@ -782,13 +791,13 @@
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
     </row>
@@ -796,13 +805,13 @@
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
     </row>
@@ -810,13 +819,13 @@
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="14"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
     </row>
@@ -824,13 +833,13 @@
       <c r="A13" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
       <c r="I13" s="4"/>
       <c r="J13" s="4"/>
     </row>
@@ -849,18 +858,18 @@
       <c r="J14" s="10"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="21" t="s">
+      <c r="A15" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="21"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="22"/>
+      <c r="J15" s="22"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
@@ -868,13 +877,13 @@
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="15"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
@@ -883,26 +892,26 @@
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="15"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="14"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="12" t="s">
         <v>15</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="23"/>
-      <c r="J18" s="15"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="I18" s="20"/>
+      <c r="J18" s="14"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
@@ -919,60 +928,60 @@
       <c r="J19" s="10"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="22"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="19"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
-      <c r="I21" s="15"/>
-      <c r="J21" s="23"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="20"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="23"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="20"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="15"/>
-      <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="15"/>
-      <c r="F23" s="15"/>
-      <c r="G23" s="15"/>
-      <c r="H23" s="15"/>
-      <c r="I23" s="15"/>
-      <c r="J23" s="23"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="20"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
@@ -986,7 +995,7 @@
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
-      <c r="J24" s="23"/>
+      <c r="J24" s="20"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
@@ -1000,7 +1009,7 @@
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
-      <c r="J25" s="23"/>
+      <c r="J25" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1013,6 +1022,33 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="10d644ba-cf16-43e8-a31a-a6f565d9c224">
+      <UserInfo>
+        <DisplayName>Helen Browne</DisplayName>
+        <AccountId>773</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <TaxCatchAll xmlns="10d644ba-cf16-43e8-a31a-a6f565d9c224" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B31D159F86750749BAD869CB65D39E6C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b52437f09c885264a74a7224ddae0bf2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94" xmlns:ns3="10d644ba-cf16-43e8-a31a-a6f565d9c224" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5a7cbcd1702d69c471f1439a09cbaf55" ns2:_="" ns3:_="">
     <xsd:import namespace="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94"/>
@@ -1267,34 +1303,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AAEB363-E0B7-4846-BB2E-A880D29866B2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="10d644ba-cf16-43e8-a31a-a6f565d9c224"/>
+    <ds:schemaRef ds:uri="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="10d644ba-cf16-43e8-a31a-a6f565d9c224">
-      <UserInfo>
-        <DisplayName>Helen Browne</DisplayName>
-        <AccountId>773</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <TaxCatchAll xmlns="10d644ba-cf16-43e8-a31a-a6f565d9c224" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5823592-756B-4A38-BF13-8C42D4724CD5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D154ECB-7BD7-4B38-A220-236438B72B0E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1311,23 +1339,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5823592-756B-4A38-BF13-8C42D4724CD5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AAEB363-E0B7-4846-BB2E-A880D29866B2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="10d644ba-cf16-43e8-a31a-a6f565d9c224"/>
-    <ds:schemaRef ds:uri="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Made ticket fully functional
</commit_message>
<xml_diff>
--- a/documentation/Time Plan.xlsx
+++ b/documentation/Time Plan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://collyer82-my.sharepoint.com/personal/25cookeg899_collyers_ac_uk/Documents/01 - Computer Science/Python Projects/Theatre-Booking/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="8_{2D523807-7404-4E18-A3A7-2E609803194E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC314E1B-3D14-4D33-B544-DD9482764C10}"/>
+  <xr:revisionPtr revIDLastSave="78" documentId="8_{2D523807-7404-4E18-A3A7-2E609803194E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5C34284-5E28-4EF5-82BE-A7058F6B0C1B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -340,7 +340,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -417,23 +417,26 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -455,6 +458,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -735,18 +742,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
@@ -995,58 +1002,58 @@
       <c r="J17" s="12"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="30"/>
-      <c r="C18" s="33" t="s">
+      <c r="B18" s="28"/>
+      <c r="C18" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="32"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
-      <c r="I18" s="30"/>
-      <c r="J18" s="30"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="28"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="31" t="s">
+      <c r="A19" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="30"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
-      <c r="H19" s="30"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="30"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="28"/>
+      <c r="J19" s="28"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="29" t="s">
+      <c r="A20" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="29"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="29"/>
-      <c r="G20" s="29"/>
-      <c r="H20" s="29"/>
-      <c r="I20" s="29"/>
-      <c r="J20" s="29"/>
+      <c r="B20" s="33"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="33"/>
+      <c r="I20" s="33"/>
+      <c r="J20" s="33"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B21" s="13"/>
-      <c r="C21" s="33" t="s">
+      <c r="C21" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="14"/>
+      <c r="D21" s="24"/>
       <c r="E21" s="14"/>
       <c r="F21" s="14"/>
       <c r="G21" s="14"/>
@@ -1191,33 +1198,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="10d644ba-cf16-43e8-a31a-a6f565d9c224">
-      <UserInfo>
-        <DisplayName>Helen Browne</DisplayName>
-        <AccountId>773</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <TaxCatchAll xmlns="10d644ba-cf16-43e8-a31a-a6f565d9c224" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B31D159F86750749BAD869CB65D39E6C" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b52437f09c885264a74a7224ddae0bf2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94" xmlns:ns3="10d644ba-cf16-43e8-a31a-a6f565d9c224" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5a7cbcd1702d69c471f1439a09cbaf55" ns2:_="" ns3:_="">
     <xsd:import namespace="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94"/>
@@ -1472,26 +1452,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AAEB363-E0B7-4846-BB2E-A880D29866B2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="10d644ba-cf16-43e8-a31a-a6f565d9c224"/>
-    <ds:schemaRef ds:uri="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5823592-756B-4A38-BF13-8C42D4724CD5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="10d644ba-cf16-43e8-a31a-a6f565d9c224">
+      <UserInfo>
+        <DisplayName>Helen Browne</DisplayName>
+        <AccountId>773</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <TaxCatchAll xmlns="10d644ba-cf16-43e8-a31a-a6f565d9c224" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D154ECB-7BD7-4B38-A220-236438B72B0E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1508,4 +1496,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5823592-756B-4A38-BF13-8C42D4724CD5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AAEB363-E0B7-4846-BB2E-A880D29866B2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="10d644ba-cf16-43e8-a31a-a6f565d9c224"/>
+    <ds:schemaRef ds:uri="9f27979c-cb1a-4f8c-bada-64f9d3ac4d94"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added admin dashboard and add event pages - still need to add content
</commit_message>
<xml_diff>
--- a/documentation/Time Plan.xlsx
+++ b/documentation/Time Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://collyer82-my.sharepoint.com/personal/25cookeg899_collyers_ac_uk/Documents/01 - Computer Science/Python Projects/Theatre-Booking/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="78" documentId="8_{2D523807-7404-4E18-A3A7-2E609803194E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5C34284-5E28-4EF5-82BE-A7058F6B0C1B}"/>
+  <xr:revisionPtr revIDLastSave="80" documentId="8_{2D523807-7404-4E18-A3A7-2E609803194E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5F05437-D146-4B3A-8312-E0686CD9494F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
   <si>
     <t>Time Plan: Design and Develop a Theatre Booking System</t>
   </si>
@@ -340,7 +340,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -436,6 +436,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1023,7 +1026,9 @@
       </c>
       <c r="B19" s="28"/>
       <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
+      <c r="D19" s="35" t="s">
+        <v>30</v>
+      </c>
       <c r="E19" s="30"/>
       <c r="F19" s="30"/>
       <c r="G19" s="30"/>

</xml_diff>

<commit_message>
Made toggle seats work with js and list
</commit_message>
<xml_diff>
--- a/documentation/Time Plan.xlsx
+++ b/documentation/Time Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://collyer82-my.sharepoint.com/personal/25cookeg899_collyers_ac_uk/Documents/01 - Computer Science/Python Projects/Theatre-Booking/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="80" documentId="8_{2D523807-7404-4E18-A3A7-2E609803194E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5F05437-D146-4B3A-8312-E0686CD9494F}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="8_{2D523807-7404-4E18-A3A7-2E609803194E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08951E6D-F1D8-4181-B20D-877F9B39DBB8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1029,7 +1029,7 @@
       <c r="D19" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="E19" s="30"/>
+      <c r="E19" s="34"/>
       <c r="F19" s="30"/>
       <c r="G19" s="30"/>
       <c r="H19" s="28"/>
@@ -1059,7 +1059,7 @@
         <v>30</v>
       </c>
       <c r="D21" s="24"/>
-      <c r="E21" s="14"/>
+      <c r="E21" s="24"/>
       <c r="F21" s="14"/>
       <c r="G21" s="14"/>
       <c r="H21" s="14"/>

</xml_diff>